<commit_message>
Complete power budget with power source, battery life, and LED loads
- Add indicator LEDs to the +5 V rail (402 mA, 502.5 mA with margin)
- Fill in the 9 V adapter power source and battery life sections
- Add regulator heat at 9 V and 12.6 V and how the budget shaped the design
- Update totals on component selection and schematic pages
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget-LiDAR.xlsx
+++ b/docs/05-Power-Budget/PowerBudget-LiDAR.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Power Budget" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Power Budget'!$A$1:$H$72</definedName>
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -934,7 +936,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1299,6 +1301,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1804,7 +1809,7 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>1.0 (10/19/2026)</t>
+          <t>1.1 (10/28/2026)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n"/>
@@ -2344,12 +2349,31 @@
     </row>
     <row r="30" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="5" t="n"/>
-      <c r="B30" s="46" t="n"/>
-      <c r="C30" s="46" t="n"/>
-      <c r="D30" s="47" t="n"/>
-      <c r="E30" s="47" t="n"/>
-      <c r="F30" s="47" t="n"/>
-      <c r="G30" s="47" t="n"/>
+      <c r="B30" s="46" t="inlineStr">
+        <is>
+          <t>Indicator LEDs (D1 power, D3/D4 debug)</t>
+        </is>
+      </c>
+      <c r="C30" s="46" t="inlineStr">
+        <is>
+          <t>Green/red LEDs, 330 R / 1 k</t>
+        </is>
+      </c>
+      <c r="D30" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +3.3 - 5V</t>
+        </is>
+      </c>
+      <c r="E30" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="47">
+        <f>E30*F30</f>
+        <v/>
+      </c>
       <c r="H30" s="47" t="inlineStr">
         <is>
           <t>mA</t>
@@ -2766,15 +2790,36 @@
       </c>
       <c r="B49" s="61" t="inlineStr">
         <is>
-          <t>Will calculate and decide as a group</t>
-        </is>
-      </c>
-      <c r="C49" s="24" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="24" t="n"/>
-      <c r="F49" s="24" t="n"/>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="68" t="n"/>
+          <t>9 V DC wall adapter</t>
+        </is>
+      </c>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>Barrel plug to fit J1 (PJ-063AH)</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 100 - 240V AC</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>9V DC</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G49" s="24">
+        <f>F49</f>
+        <v/>
+      </c>
+      <c r="H49" s="68" t="inlineStr">
+        <is>
+          <t>mA</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="69" t="n"/>
@@ -2794,15 +2839,35 @@
       </c>
       <c r="B51" s="54" t="inlineStr">
         <is>
-          <t>Will calculate and decide as a group</t>
-        </is>
-      </c>
-      <c r="C51" s="54" t="n"/>
-      <c r="D51" s="21" t="n"/>
-      <c r="E51" s="21" t="n"/>
-      <c r="F51" s="21" t="n"/>
-      <c r="G51" s="21" t="n"/>
-      <c r="H51" s="43" t="n"/>
+          <t>+5V rail (LM2940CT-5.0 input)</t>
+        </is>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>LM2940CT-5.0</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +6V - 26V</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="21">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="G51" s="21">
+        <f>E51*F51</f>
+        <v/>
+      </c>
+      <c r="H51" s="43" t="inlineStr">
+        <is>
+          <t>mA</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="144" t="n"/>
@@ -2835,8 +2900,15 @@
       <c r="D54" s="147" t="n"/>
       <c r="E54" s="147" t="n"/>
       <c r="F54" s="148" t="n"/>
-      <c r="G54" s="77" t="n"/>
-      <c r="H54" s="78" t="n"/>
+      <c r="G54" s="77">
+        <f>G49-SUM(G51:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="78" t="inlineStr">
+        <is>
+          <t>mA</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" thickBot="1">
       <c r="A55" s="11" t="n"/>
@@ -3088,14 +3160,27 @@
       <c r="A66" s="116" t="n"/>
       <c r="B66" s="46" t="inlineStr">
         <is>
-          <t>Will calculate and decide as a group</t>
-        </is>
-      </c>
-      <c r="C66" s="46" t="n"/>
-      <c r="D66" s="47" t="n"/>
+          <t>3S Li-ion pack (3 x 18650 cells, example)</t>
+        </is>
+      </c>
+      <c r="C66" s="46" t="inlineStr">
+        <is>
+          <t>3S1P 18650, 2600 mAh cells</t>
+        </is>
+      </c>
+      <c r="D66" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +9.0 - 12.6V</t>
+        </is>
+      </c>
       <c r="E66" s="47" t="n"/>
-      <c r="F66" s="47" t="n"/>
-      <c r="G66" s="47" t="n"/>
+      <c r="F66" s="47" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G66" s="47">
+        <f>G33</f>
+        <v/>
+      </c>
       <c r="H66" s="73" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" thickBot="1" thickTop="1">
@@ -3109,8 +3194,15 @@
           <t>Battery Life</t>
         </is>
       </c>
-      <c r="G67" s="121" t="n"/>
-      <c r="H67" s="122" t="n"/>
+      <c r="G67" s="159">
+        <f>F66/G66</f>
+        <v/>
+      </c>
+      <c r="H67" s="122" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" thickBot="1">
       <c r="A68" s="79" t="n"/>
@@ -3137,13 +3229,17 @@
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="154" t="inlineStr">
         <is>
-          <t>Power source selection and battery life cover the whole robot (all five subsystems), so they will be calculated and decided as a group.</t>
+          <t>Bench and testing use the 9 V DC adapter on J1 (9-12 V OK). The input current is about the same as the +5 V load because the LM2940 is a linear regulator. Battery life uses an example 3S Li-ion pack; the final robot battery is chosen as a group.</t>
         </is>
       </c>
       <c r="H70" s="155" t="n"/>
     </row>
     <row r="71" ht="48" customHeight="1" thickBot="1">
-      <c r="A71" s="156" t="n"/>
+      <c r="A71" s="156" t="inlineStr">
+        <is>
+          <t>A linear regulator wastes (Vin - 5 V) x I as heat: about 2.0 W at 9 V in and about 3.8 W at 12.6 V (full 3S pack), so U2 needs a TO-220 heatsink.</t>
+        </is>
+      </c>
       <c r="B71" s="147" t="n"/>
       <c r="C71" s="147" t="n"/>
       <c r="D71" s="147" t="n"/>
@@ -3155,7 +3251,7 @@
     <row r="72" ht="48" customHeight="1">
       <c r="A72" s="158" t="inlineStr">
         <is>
-          <t>Curiosity Nano current (100 mA) is a conservative allowance for the PIC18F57Q43 at 64 MHz plus the on-board nEDBG debugger; D500 current (290 mA) is the Waveshare/LDRobot rated working current.</t>
+          <t>Curiosity Nano current (100 mA) is a conservative allowance for the PIC18F57Q43 at 64 MHz plus the on-board nEDBG debugger; D500 current (290 mA) is the rated working current (measured 247 mA on the bench). LEDs are about 4 mA each.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update datasheet for 3S battery and fill in missing sections
- Power budget: 3S 18650 pack as source 1, 9 V adapter as source 2, 6.0 h battery life
- Component selection: power source comparison, pin table matching the schematic, MCC configuration
- New block diagram with the power path, plus draw.io source and ZIP
- Replace template BOM with the board's parts list
- Remove template appendix and old build output; fix site settings
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget-LiDAR.xlsx
+++ b/docs/05-Power-Budget/PowerBudget-LiDAR.xlsx
@@ -1809,7 +1809,7 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>1.1 (10/28/2026)</t>
+          <t>1.2 (10/28/2026)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n"/>
@@ -2790,26 +2790,26 @@
       </c>
       <c r="B49" s="61" t="inlineStr">
         <is>
-          <t>9 V DC wall adapter</t>
+          <t>3S Li-ion pack (3 x 18650 in series)</t>
         </is>
       </c>
       <c r="C49" s="24" t="inlineStr">
         <is>
-          <t>Barrel plug to fit J1 (PJ-063AH)</t>
+          <t>POWOBEST POWO18B 3000 mAh (x3)</t>
         </is>
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 100 - 240V AC</t>
+          <t xml:space="preserve"> +9.0 - 12.6V</t>
         </is>
       </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>9V DC</t>
+          <t>11.1V nom.</t>
         </is>
       </c>
       <c r="F49" s="24" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G49" s="24">
         <f>F49</f>
@@ -2924,7 +2924,7 @@
     <row r="56" ht="48" customHeight="1" thickBot="1">
       <c r="A56" s="63" t="inlineStr">
         <is>
-          <t>External Power Source 2 (unused)</t>
+          <t>External Power Source 2 (bench)</t>
         </is>
       </c>
       <c r="B56" s="64" t="inlineStr">
@@ -2977,29 +2977,30 @@
       </c>
       <c r="B57" s="61" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>9 V DC wall adapter</t>
         </is>
       </c>
       <c r="C57" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2.1 mm barrel plug (fits J1, PJ-063AH)</t>
         </is>
       </c>
       <c r="D57" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t xml:space="preserve"> 100 - 240V AC</t>
         </is>
       </c>
       <c r="E57" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9V DC</t>
         </is>
       </c>
       <c r="F57" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="24" t="n">
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="G57" s="24">
+        <f>F57</f>
+        <v/>
       </c>
       <c r="H57" s="68" t="inlineStr">
         <is>
@@ -3026,24 +3027,25 @@
       </c>
       <c r="B59" s="54" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>+5V rail (LM2940CT-5.0 input)</t>
         </is>
       </c>
       <c r="C59" s="54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>LM2940CT-5.0</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t xml:space="preserve"> +6V - 26V</t>
         </is>
       </c>
       <c r="E59" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F59" s="21">
+        <f>G33</f>
+        <v/>
       </c>
       <c r="G59" s="21">
         <f>E59*F59</f>
@@ -3160,12 +3162,12 @@
       <c r="A66" s="116" t="n"/>
       <c r="B66" s="46" t="inlineStr">
         <is>
-          <t>3S Li-ion pack (3 x 18650 cells, example)</t>
+          <t>3S Li-ion pack (3 x 18650 in series)</t>
         </is>
       </c>
       <c r="C66" s="46" t="inlineStr">
         <is>
-          <t>3S1P 18650, 2600 mAh cells</t>
+          <t>POWOBEST POWO18B 3000 mAh (x3)</t>
         </is>
       </c>
       <c r="D66" s="47" t="inlineStr">
@@ -3175,7 +3177,7 @@
       </c>
       <c r="E66" s="47" t="n"/>
       <c r="F66" s="47" t="n">
-        <v>2600</v>
+        <v>3000</v>
       </c>
       <c r="G66" s="47">
         <f>G33</f>
@@ -3229,7 +3231,7 @@
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="154" t="inlineStr">
         <is>
-          <t>Bench and testing use the 9 V DC adapter on J1 (9-12 V OK). The input current is about the same as the +5 V load because the LM2940 is a linear regulator. Battery life uses an example 3S Li-ion pack; the final robot battery is chosen as a group.</t>
+          <t>On the robot, the board runs from a 3S pack of 3.7 V 18650 cells in series (9.0 V empty, 11.1 V nominal, 12.6 V full), plugged into J1. On the bench, a 9 V adapter plugs into J1 instead. Only one source is connected at a time. A linear regulator draws about the same current from its input as it delivers, so each source supplies about 502.5 mA. Battery max current assumes 1C (3000 mA) continuous because no cell datasheet is available.</t>
         </is>
       </c>
       <c r="H70" s="155" t="n"/>
@@ -3237,7 +3239,7 @@
     <row r="71" ht="48" customHeight="1" thickBot="1">
       <c r="A71" s="156" t="inlineStr">
         <is>
-          <t>A linear regulator wastes (Vin - 5 V) x I as heat: about 2.0 W at 9 V in and about 3.8 W at 12.6 V (full 3S pack), so U2 needs a TO-220 heatsink.</t>
+          <t>Regulator heat is (Vin - 5 V) x I: about 2.0 W at 9 V and about 3.8 W at 12.6 V (full pack), so U2 needs a TO-220 heatsink. Cells are charged one at a time with TP4056 modules, removed from the series pack.</t>
         </is>
       </c>
       <c r="B71" s="147" t="n"/>

</xml_diff>